<commit_message>
chingo de cambios en el admin
</commit_message>
<xml_diff>
--- a/bd/producto.xlsx
+++ b/bd/producto.xlsx
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>165777</v>
+        <v>200</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -503,10 +503,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61763</v>
+        <v>60</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -531,14 +531,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kllklk</t>
+          <t>puro de corazon</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>300</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -548,8 +548,8 @@
           <t>img/producto_3.jpg</t>
         </is>
       </c>
-      <c r="H4" t="n">
-        <v>1</v>
+      <c r="H4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>